<commit_message>
N-min lab file: remove rows from other projects analysed in the same runs
The pipeline already dropped these rows; all outputs are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/soil/nmin/Yale_inorgN_2026.xlsx
+++ b/data/raw/soil/nmin/Yale_inorgN_2026.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="213">
   <si>
     <t>Sample ID</t>
   </si>
@@ -36,36 +36,6 @@
     <t>mg N-NH4/L</t>
   </si>
   <si>
-    <t>EU PO 10/2025 _SRS5 90</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS5 45</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS5 15</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS5 0</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS5 surface</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS6 90</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS6 45</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS6 15</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS6 0</t>
-  </si>
-  <si>
-    <t>EU PO 10/2025 _SRS6 surface</t>
-  </si>
-  <si>
     <t>T3_blank</t>
   </si>
   <si>
@@ -694,36 +664,6 @@
   </si>
   <si>
     <t>183_N min 3_P1 T1_A</t>
-  </si>
-  <si>
-    <t>CP40 90</t>
-  </si>
-  <si>
-    <t>CP40 45</t>
-  </si>
-  <si>
-    <t>CP40 15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CP40 C </t>
-  </si>
-  <si>
-    <t>CP40 surface</t>
-  </si>
-  <si>
-    <t>BL60 90</t>
-  </si>
-  <si>
-    <t>BL60 45</t>
-  </si>
-  <si>
-    <t>BL60 15</t>
-  </si>
-  <si>
-    <t>BL60 0</t>
-  </si>
-  <si>
-    <t>BL60 surface</t>
   </si>
 </sst>
 </file>
@@ -1111,7 +1051,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB1E098C-6A9B-48BD-967D-1B10FBF85871}">
-  <dimension ref="A1:D240"/>
+  <dimension ref="A1:D220"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="29.7265625" customWidth="1"/>
@@ -1142,142 +1082,142 @@
         <v>3</v>
       </c>
       <c r="B2" s="2">
-        <v>-0.29612539999999987</v>
+        <v>-0.25222069999999985</v>
       </c>
       <c r="C2" s="2">
-        <v>-0.43353084999999991</v>
+        <v>1.0323983000000001</v>
       </c>
       <c r="D2" s="3"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3" s="2">
-        <v>-0.2847426999999999</v>
+        <v>-0.23433359999999992</v>
       </c>
       <c r="C3" s="2">
-        <v>-0.40670019999999996</v>
+        <v>1.3755054000000002</v>
       </c>
       <c r="D3" s="3"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A4" s="1" t="s">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2">
-        <v>-0.27661219999999986</v>
+        <v>-0.25059459999999989</v>
       </c>
       <c r="C4" s="2">
-        <v>-0.41320460000000003</v>
+        <v>0.69823475000000013</v>
       </c>
       <c r="D4" s="3"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B5" s="2">
-        <v>-0.24734239999999985</v>
+        <v>2.0308237000000005</v>
       </c>
       <c r="C5" s="2">
-        <v>-0.34084314999999998</v>
+        <v>1.5690113000000001</v>
       </c>
       <c r="D5" s="3"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B6" s="2">
-        <v>-0.22295090000000006</v>
+        <v>1.4893323999999999</v>
       </c>
       <c r="C6" s="2">
-        <v>-0.40019579999999988</v>
+        <v>0.75596130000000006</v>
       </c>
       <c r="D6" s="3"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B7" s="2">
-        <v>-0.30913419999999991</v>
+        <v>1.2925743000000001</v>
       </c>
       <c r="C7" s="2">
-        <v>-0.46280064999999992</v>
+        <v>0.96898040000000019</v>
       </c>
       <c r="D7" s="3"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="B8" s="2">
-        <v>-0.30913419999999991</v>
+        <v>2.1812379500000008</v>
       </c>
       <c r="C8" s="2">
-        <v>-0.50914449999999989</v>
+        <v>0.50879410000000025</v>
       </c>
       <c r="D8" s="3"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B9" s="2">
-        <v>-0.31401249999999992</v>
+        <v>1.4275405999999999</v>
       </c>
       <c r="C9" s="2">
-        <v>-0.50101399999999985</v>
+        <v>1.1819994999999999</v>
       </c>
       <c r="D9" s="3"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10" s="2">
-        <v>-0.25384679999999993</v>
+        <v>1.9958625500000005</v>
       </c>
       <c r="C10" s="2">
-        <v>-0.47011809999999987</v>
+        <v>1.2990787000000004</v>
       </c>
       <c r="D10" s="3"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11" s="2">
-        <v>-0.24083799999999989</v>
+        <v>1.0397157500000003</v>
       </c>
       <c r="C11" s="2">
-        <v>-0.40019579999999988</v>
+        <v>0.43561960000000011</v>
       </c>
       <c r="D11" s="3"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A12" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12" s="2">
-        <v>-0.25222069999999985</v>
+        <v>1.3917663999999998</v>
       </c>
       <c r="C12" s="2">
-        <v>1.0323983000000001</v>
+        <v>1.3007048000000001</v>
       </c>
       <c r="D12" s="3"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B13" s="2">
-        <v>-0.23433359999999992</v>
+        <v>0.90231030000000034</v>
       </c>
       <c r="C13" s="2">
-        <v>1.3755054000000002</v>
+        <v>1.4933976500000004</v>
       </c>
       <c r="D13" s="3"/>
     </row>
@@ -1286,10 +1226,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="2">
-        <v>-0.25059459999999989</v>
+        <v>0.68847815000000012</v>
       </c>
       <c r="C14" s="2">
-        <v>0.69823475000000013</v>
+        <v>1.0958162000000002</v>
       </c>
       <c r="D14" s="3"/>
     </row>
@@ -1298,10 +1238,10 @@
         <v>14</v>
       </c>
       <c r="B15" s="2">
-        <v>2.0308237000000005</v>
+        <v>4.1179230500000008</v>
       </c>
       <c r="C15" s="2">
-        <v>1.5690113000000001</v>
+        <v>0.91369300000000009</v>
       </c>
       <c r="D15" s="3"/>
     </row>
@@ -1310,10 +1250,10 @@
         <v>15</v>
       </c>
       <c r="B16" s="2">
-        <v>1.4893323999999999</v>
+        <v>5.2082230999999997</v>
       </c>
       <c r="C16" s="2">
-        <v>0.75596130000000006</v>
+        <v>2.1934337000000004</v>
       </c>
       <c r="D16" s="3"/>
     </row>
@@ -1322,10 +1262,10 @@
         <v>16</v>
       </c>
       <c r="B17" s="2">
-        <v>1.2925743000000001</v>
+        <v>1.8885399500000002</v>
       </c>
       <c r="C17" s="2">
-        <v>0.96898040000000019</v>
+        <v>1.1494775000000002</v>
       </c>
       <c r="D17" s="3"/>
     </row>
@@ -1334,10 +1274,10 @@
         <v>17</v>
       </c>
       <c r="B18" s="2">
-        <v>2.1812379500000008</v>
+        <v>2.5349147000000003</v>
       </c>
       <c r="C18" s="2">
-        <v>0.50879410000000025</v>
+        <v>1.1641124</v>
       </c>
       <c r="D18" s="3"/>
     </row>
@@ -1346,10 +1286,10 @@
         <v>18</v>
       </c>
       <c r="B19" s="2">
-        <v>1.4275405999999999</v>
+        <v>1.7934131000000004</v>
       </c>
       <c r="C19" s="2">
-        <v>1.1819994999999999</v>
+        <v>1.1421600500000002</v>
       </c>
       <c r="D19" s="3"/>
     </row>
@@ -1358,10 +1298,10 @@
         <v>19</v>
       </c>
       <c r="B20" s="2">
-        <v>1.9958625500000005</v>
+        <v>1.9576491999999996</v>
       </c>
       <c r="C20" s="2">
-        <v>1.2990787000000004</v>
+        <v>3.1040497</v>
       </c>
       <c r="D20" s="3"/>
     </row>
@@ -1370,10 +1310,10 @@
         <v>20</v>
       </c>
       <c r="B21" s="2">
-        <v>1.0397157500000003</v>
+        <v>2.28368225</v>
       </c>
       <c r="C21" s="2">
-        <v>0.43561960000000011</v>
+        <v>2.2909997000000004</v>
       </c>
       <c r="D21" s="3"/>
     </row>
@@ -1382,22 +1322,22 @@
         <v>21</v>
       </c>
       <c r="B22" s="2">
-        <v>1.3917663999999998</v>
+        <v>2.4958882999999998</v>
       </c>
       <c r="C22" s="2">
-        <v>1.3007048000000001</v>
+        <v>0.7982399</v>
       </c>
       <c r="D22" s="3"/>
     </row>
-    <row r="23" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B23" s="2">
-        <v>0.90231030000000034</v>
+        <v>1.0445940500000004</v>
       </c>
       <c r="C23" s="2">
-        <v>1.4933976500000004</v>
+        <v>1.6421858000000005</v>
       </c>
       <c r="D23" s="3"/>
     </row>
@@ -1406,10 +1346,10 @@
         <v>23</v>
       </c>
       <c r="B24" s="2">
-        <v>0.68847815000000012</v>
+        <v>1.0063807000000002</v>
       </c>
       <c r="C24" s="2">
-        <v>1.0958162000000002</v>
+        <v>2.0064322000000003</v>
       </c>
       <c r="D24" s="3"/>
     </row>
@@ -1418,10 +1358,10 @@
         <v>24</v>
       </c>
       <c r="B25" s="2">
-        <v>4.1179230500000008</v>
+        <v>1.7527606000000007</v>
       </c>
       <c r="C25" s="2">
-        <v>0.91369300000000009</v>
+        <v>1.7446301000000006</v>
       </c>
       <c r="D25" s="3"/>
     </row>
@@ -1430,10 +1370,10 @@
         <v>25</v>
       </c>
       <c r="B26" s="2">
-        <v>5.2082230999999997</v>
+        <v>2.4601141000000002</v>
       </c>
       <c r="C26" s="2">
-        <v>2.1934337000000004</v>
+        <v>1.8340655999999997</v>
       </c>
       <c r="D26" s="3"/>
     </row>
@@ -1442,10 +1382,10 @@
         <v>26</v>
       </c>
       <c r="B27" s="2">
-        <v>1.8885399500000002</v>
+        <v>2.7934646000000005</v>
       </c>
       <c r="C27" s="2">
-        <v>1.1494775000000002</v>
+        <v>0.71205660000000015</v>
       </c>
       <c r="D27" s="3"/>
     </row>
@@ -1454,10 +1394,10 @@
         <v>27</v>
       </c>
       <c r="B28" s="2">
-        <v>2.5349147000000003</v>
+        <v>3.8292903000000003</v>
       </c>
       <c r="C28" s="2">
-        <v>1.1641124</v>
+        <v>1.4129057</v>
       </c>
       <c r="D28" s="3"/>
     </row>
@@ -1466,10 +1406,10 @@
         <v>28</v>
       </c>
       <c r="B29" s="2">
-        <v>1.7934131000000004</v>
+        <v>1.7023515000000007</v>
       </c>
       <c r="C29" s="2">
-        <v>1.1421600500000002</v>
+        <v>0.61123839999999996</v>
       </c>
       <c r="D29" s="3"/>
     </row>
@@ -1478,10 +1418,10 @@
         <v>29</v>
       </c>
       <c r="B30" s="2">
-        <v>1.9576491999999996</v>
+        <v>1.2177737000000004</v>
       </c>
       <c r="C30" s="2">
-        <v>3.1040497</v>
+        <v>0.71856100000000023</v>
       </c>
       <c r="D30" s="3"/>
     </row>
@@ -1490,10 +1430,10 @@
         <v>30</v>
       </c>
       <c r="B31" s="2">
-        <v>2.28368225</v>
+        <v>4.0740183500000002</v>
       </c>
       <c r="C31" s="2">
-        <v>2.2909997000000004</v>
+        <v>0.5705859000000002</v>
       </c>
       <c r="D31" s="3"/>
     </row>
@@ -1502,10 +1442,10 @@
         <v>31</v>
       </c>
       <c r="B32" s="2">
-        <v>2.4958882999999998</v>
+        <v>4.7691761000000001</v>
       </c>
       <c r="C32" s="2">
-        <v>0.7982399</v>
+        <v>1.3820098000000001</v>
       </c>
       <c r="D32" s="3"/>
     </row>
@@ -1514,10 +1454,10 @@
         <v>32</v>
       </c>
       <c r="B33" s="2">
-        <v>1.0445940500000004</v>
+        <v>1.9495187</v>
       </c>
       <c r="C33" s="2">
-        <v>1.6421858000000005</v>
+        <v>0.48277650000000016</v>
       </c>
       <c r="D33" s="3"/>
     </row>
@@ -1526,10 +1466,10 @@
         <v>33</v>
       </c>
       <c r="B34" s="2">
-        <v>1.0063807000000002</v>
+        <v>1.6299900500000004</v>
       </c>
       <c r="C34" s="2">
-        <v>2.0064322000000003</v>
+        <v>0.96247600000000033</v>
       </c>
       <c r="D34" s="3"/>
     </row>
@@ -1538,142 +1478,142 @@
         <v>34</v>
       </c>
       <c r="B35" s="2">
-        <v>1.7527606000000007</v>
+        <v>-0.26035119999999989</v>
       </c>
       <c r="C35" s="2">
-        <v>1.7446301000000006</v>
+        <v>1.0161373000000002</v>
       </c>
       <c r="D35" s="3"/>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B36" s="2">
-        <v>2.4601141000000002</v>
+        <v>-0.25709899999999986</v>
       </c>
       <c r="C36" s="2">
-        <v>1.8340655999999997</v>
+        <v>0.81450090000000008</v>
       </c>
       <c r="D36" s="3"/>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A37" s="1" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B37" s="2">
-        <v>2.7934646000000005</v>
+        <v>-0.25384679999999993</v>
       </c>
       <c r="C37" s="2">
-        <v>0.71205660000000015</v>
+        <v>1.2259042000000004</v>
       </c>
       <c r="D37" s="3"/>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A38" s="1" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B38" s="2">
-        <v>3.8292903000000003</v>
+        <v>5.6911747999999998</v>
       </c>
       <c r="C38" s="2">
-        <v>1.4129057</v>
+        <v>0.98036310000000038</v>
       </c>
       <c r="D38" s="3"/>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B39" s="2">
-        <v>1.7023515000000007</v>
+        <v>6.7302527000000003</v>
       </c>
       <c r="C39" s="2">
-        <v>0.61123839999999996</v>
+        <v>1.0649203000000003</v>
       </c>
       <c r="D39" s="3"/>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B40" s="2">
-        <v>1.2177737000000004</v>
+        <v>5.1106571000000001</v>
       </c>
       <c r="C40" s="2">
-        <v>0.71856100000000023</v>
+        <v>0.92507570000000028</v>
       </c>
       <c r="D40" s="3"/>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A41" s="1" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B41" s="2">
-        <v>4.0740183500000002</v>
+        <v>9.354778099999999</v>
       </c>
       <c r="C41" s="2">
-        <v>0.5705859000000002</v>
+        <v>1.1567949500000001</v>
       </c>
       <c r="D41" s="3"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A42" s="1" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B42" s="2">
-        <v>4.7691761000000001</v>
+        <v>3.4544742500000005</v>
       </c>
       <c r="C42" s="2">
-        <v>1.3820098000000001</v>
+        <v>1.0600420000000006</v>
       </c>
       <c r="D42" s="3"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A43" s="1" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B43" s="2">
-        <v>1.9495187</v>
+        <v>2.9739617000000007</v>
       </c>
       <c r="C43" s="2">
-        <v>0.48277650000000016</v>
+        <v>1.1088250000000004</v>
       </c>
       <c r="D43" s="3"/>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A44" s="1" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B44" s="2">
-        <v>1.6299900500000004</v>
+        <v>-0.21969870000000002</v>
       </c>
       <c r="C44" s="2">
-        <v>0.96247600000000033</v>
+        <v>1.739751800000001</v>
       </c>
       <c r="D44" s="3"/>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A45" s="1" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B45" s="2">
-        <v>-0.26035119999999989</v>
+        <v>14.572933000000004</v>
       </c>
       <c r="C45" s="2">
-        <v>1.0161373000000002</v>
+        <v>1.4348580500000003</v>
       </c>
       <c r="D45" s="3"/>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A46" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B46" s="2">
-        <v>-0.25709899999999986</v>
+        <v>5.9367159000000003</v>
       </c>
       <c r="C46" s="2">
-        <v>0.81450090000000008</v>
+        <v>1.1462252999999998</v>
       </c>
       <c r="D46" s="3"/>
     </row>
@@ -1682,10 +1622,10 @@
         <v>44</v>
       </c>
       <c r="B47" s="2">
-        <v>-0.25384679999999993</v>
+        <v>5.2456234000000004</v>
       </c>
       <c r="C47" s="2">
-        <v>1.2259042000000004</v>
+        <v>1.1494775000000002</v>
       </c>
       <c r="D47" s="3"/>
     </row>
@@ -1694,22 +1634,22 @@
         <v>45</v>
       </c>
       <c r="B48" s="2">
-        <v>5.6911747999999998</v>
+        <v>9.5531623000000021</v>
       </c>
       <c r="C48" s="2">
-        <v>0.98036310000000038</v>
+        <v>1.3608704999999999</v>
       </c>
       <c r="D48" s="3"/>
     </row>
-    <row r="49" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B49" s="2">
-        <v>6.7302527000000003</v>
+        <v>4.8634899000000011</v>
       </c>
       <c r="C49" s="2">
-        <v>1.0649203000000003</v>
+        <v>0.99825019999999998</v>
       </c>
       <c r="D49" s="3"/>
     </row>
@@ -1718,10 +1658,10 @@
         <v>47</v>
       </c>
       <c r="B50" s="2">
-        <v>5.1106571000000001</v>
+        <v>13.523285450000001</v>
       </c>
       <c r="C50" s="2">
-        <v>0.92507570000000028</v>
+        <v>1.3202180000000001</v>
       </c>
       <c r="D50" s="3"/>
     </row>
@@ -1730,10 +1670,10 @@
         <v>48</v>
       </c>
       <c r="B51" s="2">
-        <v>9.354778099999999</v>
+        <v>1.9722840999999995</v>
       </c>
       <c r="C51" s="2">
-        <v>1.1567949500000001</v>
+        <v>1.4291667000000001</v>
       </c>
       <c r="D51" s="3"/>
     </row>
@@ -1742,10 +1682,10 @@
         <v>49</v>
       </c>
       <c r="B52" s="2">
-        <v>3.4544742500000005</v>
+        <v>8.2978131000000008</v>
       </c>
       <c r="C52" s="2">
-        <v>1.0600420000000006</v>
+        <v>1.7316213</v>
       </c>
       <c r="D52" s="3"/>
     </row>
@@ -1754,10 +1694,10 @@
         <v>50</v>
       </c>
       <c r="B53" s="2">
-        <v>2.9739617000000007</v>
+        <v>3.8959603999999999</v>
       </c>
       <c r="C53" s="2">
-        <v>1.1088250000000004</v>
+        <v>0.91206690000000035</v>
       </c>
       <c r="D53" s="3"/>
     </row>
@@ -1766,10 +1706,10 @@
         <v>51</v>
       </c>
       <c r="B54" s="2">
-        <v>-0.21969870000000002</v>
+        <v>4.0179179000000014</v>
       </c>
       <c r="C54" s="2">
-        <v>1.739751800000001</v>
+        <v>1.5413676000000001</v>
       </c>
       <c r="D54" s="3"/>
     </row>
@@ -1778,10 +1718,10 @@
         <v>52</v>
       </c>
       <c r="B55" s="2">
-        <v>14.572933000000004</v>
+        <v>1.4421755000000003</v>
       </c>
       <c r="C55" s="2">
-        <v>1.4348580500000003</v>
+        <v>2.1495290000000002</v>
       </c>
       <c r="D55" s="3"/>
     </row>
@@ -1790,10 +1730,10 @@
         <v>53</v>
       </c>
       <c r="B56" s="2">
-        <v>5.9367159000000003</v>
+        <v>5.1285442000000012</v>
       </c>
       <c r="C56" s="2">
-        <v>1.1462252999999998</v>
+        <v>1.6226726000000005</v>
       </c>
       <c r="D56" s="3"/>
     </row>
@@ -1802,130 +1742,130 @@
         <v>54</v>
       </c>
       <c r="B57" s="2">
-        <v>5.2456234000000004</v>
+        <v>7.0001853000000009</v>
       </c>
       <c r="C57" s="2">
-        <v>1.1494775000000002</v>
+        <v>1.3023309000000003</v>
       </c>
       <c r="D57" s="3"/>
     </row>
     <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B58" s="2">
-        <v>9.5531623000000021</v>
+        <v>7.1514125999999987</v>
       </c>
       <c r="C58" s="2">
-        <v>1.3608704999999999</v>
+        <v>1.3088353000000001</v>
       </c>
       <c r="D58" s="3"/>
     </row>
     <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B59" s="2">
-        <v>4.8634899000000011</v>
+        <v>7.1936912</v>
       </c>
       <c r="C59" s="2">
-        <v>0.99825019999999998</v>
+        <v>1.0096329000000004</v>
       </c>
       <c r="D59" s="3"/>
     </row>
     <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B60" s="2">
-        <v>13.523285450000001</v>
+        <v>7.1221428000000024</v>
       </c>
       <c r="C60" s="2">
-        <v>1.3202180000000001</v>
+        <v>0.75433520000000032</v>
       </c>
       <c r="D60" s="3"/>
     </row>
     <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B61" s="2">
-        <v>1.9722840999999995</v>
+        <v>4.5480264999999997</v>
       </c>
       <c r="C61" s="2">
-        <v>1.4291667000000001</v>
+        <v>1.3868881000000002</v>
       </c>
       <c r="D61" s="3"/>
     </row>
     <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B62" s="2">
-        <v>8.2978131000000008</v>
+        <v>6.969289400000001</v>
       </c>
       <c r="C62" s="2">
-        <v>1.7316213</v>
+        <v>1.7722738000000007</v>
       </c>
       <c r="D62" s="3"/>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B63" s="2">
-        <v>3.8959603999999999</v>
+        <v>8.4685535999999999</v>
       </c>
       <c r="C63" s="2">
-        <v>0.91206690000000035</v>
+        <v>1.9381359999999996</v>
       </c>
       <c r="D63" s="3"/>
     </row>
     <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B64" s="2">
-        <v>4.0179179000000014</v>
+        <v>6.005012100000001</v>
       </c>
       <c r="C64" s="2">
-        <v>1.5413676000000001</v>
+        <v>2.1641639000000001</v>
       </c>
       <c r="D64" s="3"/>
     </row>
     <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B65" s="2">
-        <v>1.4421755000000003</v>
+        <v>5.9562290999999998</v>
       </c>
       <c r="C65" s="2">
-        <v>2.1495290000000002</v>
+        <v>0.89580590000000004</v>
       </c>
       <c r="D65" s="3"/>
     </row>
     <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B66" s="2">
-        <v>5.1285442000000012</v>
+        <v>2.9251787000000005</v>
       </c>
       <c r="C66" s="2">
-        <v>1.6226726000000005</v>
+        <v>1.1616732500000002</v>
       </c>
       <c r="D66" s="3"/>
     </row>
     <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B67" s="2">
-        <v>7.0001853000000009</v>
+        <v>2.9715225500000004</v>
       </c>
       <c r="C67" s="2">
-        <v>1.3023309000000003</v>
+        <v>1.5665721499999998</v>
       </c>
       <c r="D67" s="3"/>
     </row>
@@ -1934,10 +1874,10 @@
         <v>64</v>
       </c>
       <c r="B68" s="2">
-        <v>7.1514125999999987</v>
+        <v>10.936973400000001</v>
       </c>
       <c r="C68" s="2">
-        <v>1.3088353000000001</v>
+        <v>1.4714453000000001</v>
       </c>
       <c r="D68" s="3"/>
     </row>
@@ -1946,10 +1886,10 @@
         <v>65</v>
       </c>
       <c r="B69" s="2">
-        <v>7.1936912</v>
+        <v>11.232923600000003</v>
       </c>
       <c r="C69" s="2">
-        <v>1.0096329000000004</v>
+        <v>1.0543506499999999</v>
       </c>
       <c r="D69" s="3"/>
     </row>
@@ -1958,10 +1898,10 @@
         <v>66</v>
       </c>
       <c r="B70" s="2">
-        <v>7.1221428000000024</v>
+        <v>7.8620183000000008</v>
       </c>
       <c r="C70" s="2">
-        <v>0.75433520000000032</v>
+        <v>1.5202283000000003</v>
       </c>
       <c r="D70" s="3"/>
     </row>
@@ -1970,10 +1910,10 @@
         <v>67</v>
       </c>
       <c r="B71" s="2">
-        <v>4.5480264999999997</v>
+        <v>5.2448103499999998</v>
       </c>
       <c r="C71" s="2">
-        <v>1.3868881000000002</v>
+        <v>1.19094305</v>
       </c>
       <c r="D71" s="3"/>
     </row>
@@ -1982,10 +1922,10 @@
         <v>68</v>
       </c>
       <c r="B72" s="2">
-        <v>6.969289400000001</v>
+        <v>8.3953790999999995</v>
       </c>
       <c r="C72" s="2">
-        <v>1.7722738000000007</v>
+        <v>3.5073224999999999</v>
       </c>
       <c r="D72" s="3"/>
     </row>
@@ -1994,10 +1934,10 @@
         <v>69</v>
       </c>
       <c r="B73" s="2">
-        <v>8.4685535999999999</v>
+        <v>1.2437912999999998</v>
       </c>
       <c r="C73" s="2">
-        <v>1.9381359999999996</v>
+        <v>14.962383950000001</v>
       </c>
       <c r="D73" s="3"/>
     </row>
@@ -2006,10 +1946,10 @@
         <v>70</v>
       </c>
       <c r="B74" s="2">
-        <v>6.005012100000001</v>
+        <v>0.58847300000000002</v>
       </c>
       <c r="C74" s="2">
-        <v>2.1641639000000001</v>
+        <v>16.337251500000001</v>
       </c>
       <c r="D74" s="3"/>
     </row>
@@ -2018,10 +1958,10 @@
         <v>71</v>
       </c>
       <c r="B75" s="2">
-        <v>5.9562290999999998</v>
+        <v>-2.9444999999999832E-2</v>
       </c>
       <c r="C75" s="2">
-        <v>0.89580590000000004</v>
+        <v>17.028344000000001</v>
       </c>
       <c r="D75" s="3"/>
     </row>
@@ -2030,10 +1970,10 @@
         <v>72</v>
       </c>
       <c r="B76" s="2">
-        <v>2.9251787000000005</v>
+        <v>-4.407989999999995E-2</v>
       </c>
       <c r="C76" s="2">
-        <v>1.1616732500000002</v>
+        <v>17.142171000000001</v>
       </c>
       <c r="D76" s="3"/>
     </row>
@@ -2041,11 +1981,11 @@
       <c r="A77" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="B77" s="2">
-        <v>2.9715225500000004</v>
+      <c r="B77" s="4">
+        <v>0.14129550000000024</v>
       </c>
       <c r="C77" s="2">
-        <v>1.5665721499999998</v>
+        <v>16.677106400000003</v>
       </c>
       <c r="D77" s="3"/>
     </row>
@@ -2053,11 +1993,11 @@
       <c r="A78" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="B78" s="2">
-        <v>10.936973400000001</v>
+      <c r="B78" s="4">
+        <v>-9.4488999999999823E-2</v>
       </c>
       <c r="C78" s="2">
-        <v>1.4714453000000001</v>
+        <v>16.829959800000001</v>
       </c>
       <c r="D78" s="3"/>
     </row>
@@ -2065,11 +2005,11 @@
       <c r="A79" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="B79" s="2">
-        <v>11.232923600000003</v>
+      <c r="B79" s="4">
+        <v>16.15025</v>
       </c>
       <c r="C79" s="2">
-        <v>1.0543506499999999</v>
+        <v>2.3950701000000008</v>
       </c>
       <c r="D79" s="3"/>
     </row>
@@ -2077,11 +2017,11 @@
       <c r="A80" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="B80" s="2">
-        <v>7.8620183000000008</v>
+      <c r="B80" s="4">
+        <v>15.906335000000002</v>
       </c>
       <c r="C80" s="2">
-        <v>1.5202283000000003</v>
+        <v>6.7375701500000007</v>
       </c>
       <c r="D80" s="3"/>
     </row>
@@ -2089,11 +2029,11 @@
       <c r="A81" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="B81" s="2">
-        <v>5.2448103499999998</v>
+      <c r="B81" s="4">
+        <v>-0.13351539999999984</v>
       </c>
       <c r="C81" s="2">
-        <v>1.19094305</v>
+        <v>16.444574100000004</v>
       </c>
       <c r="D81" s="3"/>
     </row>
@@ -2101,11 +2041,11 @@
       <c r="A82" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="B82" s="2">
-        <v>8.3953790999999995</v>
+      <c r="B82" s="4">
+        <v>-0.1611591</v>
       </c>
       <c r="C82" s="2">
-        <v>3.5073224999999999</v>
+        <v>17.242989200000004</v>
       </c>
       <c r="D82" s="3"/>
     </row>
@@ -2113,11 +2053,11 @@
       <c r="A83" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B83" s="2">
-        <v>1.2437912999999998</v>
+      <c r="B83" s="4">
+        <v>-0.1562808</v>
       </c>
       <c r="C83" s="2">
-        <v>14.962383950000001</v>
+        <v>16.888499400000001</v>
       </c>
       <c r="D83" s="3"/>
     </row>
@@ -2126,10 +2066,10 @@
         <v>80</v>
       </c>
       <c r="B84" s="2">
-        <v>0.58847300000000002</v>
+        <v>-0.14977640000000003</v>
       </c>
       <c r="C84" s="2">
-        <v>16.337251500000001</v>
+        <v>16.691741299999997</v>
       </c>
       <c r="D84" s="3"/>
     </row>
@@ -2138,10 +2078,10 @@
         <v>81</v>
       </c>
       <c r="B85" s="2">
-        <v>-2.9444999999999832E-2</v>
+        <v>4.0455616000000001</v>
       </c>
       <c r="C85" s="2">
-        <v>17.028344000000001</v>
+        <v>9.0100449000000005</v>
       </c>
       <c r="D85" s="3"/>
     </row>
@@ -2150,10 +2090,10 @@
         <v>82</v>
       </c>
       <c r="B86" s="2">
-        <v>-4.407989999999995E-2</v>
+        <v>1.5348632000000002</v>
       </c>
       <c r="C86" s="2">
-        <v>17.142171000000001</v>
+        <v>3.8601862000000002</v>
       </c>
       <c r="D86" s="3"/>
     </row>
@@ -2161,11 +2101,11 @@
       <c r="A87" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="B87" s="4">
-        <v>0.14129550000000024</v>
+      <c r="B87" s="2">
+        <v>1.7080428500000004</v>
       </c>
       <c r="C87" s="2">
-        <v>16.677106400000003</v>
+        <v>2.6178458</v>
       </c>
       <c r="D87" s="3"/>
     </row>
@@ -2173,11 +2113,11 @@
       <c r="A88" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="B88" s="4">
-        <v>-9.4488999999999823E-2</v>
+      <c r="B88" s="2">
+        <v>1.9999278000000005</v>
       </c>
       <c r="C88" s="2">
-        <v>16.829959800000001</v>
+        <v>2.2544124500000002</v>
       </c>
       <c r="D88" s="3"/>
     </row>
@@ -2185,11 +2125,11 @@
       <c r="A89" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="B89" s="4">
-        <v>16.15025</v>
+      <c r="B89" s="2">
+        <v>2.1812379500000008</v>
       </c>
       <c r="C89" s="2">
-        <v>2.3950701000000008</v>
+        <v>2.8983480500000005</v>
       </c>
       <c r="D89" s="3"/>
     </row>
@@ -2197,167 +2137,167 @@
       <c r="A90" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="B90" s="4">
-        <v>15.906335000000002</v>
+      <c r="B90" s="2">
+        <v>-0.27335999999999994</v>
       </c>
       <c r="C90" s="2">
-        <v>6.7375701500000007</v>
+        <v>1.3665618500000005</v>
       </c>
       <c r="D90" s="3"/>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="B91" s="4">
-        <v>-0.13351539999999984</v>
+        <v>86</v>
+      </c>
+      <c r="B91" s="2">
+        <v>-0.25709899999999986</v>
       </c>
       <c r="C91" s="2">
-        <v>16.444574100000004</v>
+        <v>1.3177788500000003</v>
       </c>
       <c r="D91" s="3"/>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B92" s="4">
-        <v>-0.1611591</v>
+        <v>86</v>
+      </c>
+      <c r="B92" s="2">
+        <v>-0.2749860999999999</v>
       </c>
       <c r="C92" s="2">
-        <v>17.242989200000004</v>
+        <v>1.2584262000000002</v>
       </c>
       <c r="D92" s="3"/>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="B93" s="4">
-        <v>-0.1562808</v>
+        <v>87</v>
+      </c>
+      <c r="B93" s="2">
+        <v>-0.30750809999999995</v>
       </c>
       <c r="C93" s="2">
-        <v>16.888499400000001</v>
+        <v>0.10308215000000009</v>
       </c>
       <c r="D93" s="3"/>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B94" s="2">
-        <v>-0.14977640000000003</v>
+        <v>-0.26279034999999984</v>
       </c>
       <c r="C94" s="2">
-        <v>16.691741299999997</v>
+        <v>1.2909482000000003</v>
       </c>
       <c r="D94" s="3"/>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B95" s="2">
-        <v>4.0455616000000001</v>
+        <v>1.385262</v>
       </c>
       <c r="C95" s="2">
-        <v>9.0100449000000005</v>
+        <v>2.4227137999999999</v>
       </c>
       <c r="D95" s="3"/>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B96" s="2">
-        <v>1.5348632000000002</v>
+        <v>1.1315904000000003</v>
       </c>
       <c r="C96" s="2">
-        <v>3.8601862000000002</v>
+        <v>2.4145833000000003</v>
       </c>
       <c r="D96" s="3"/>
     </row>
     <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B97" s="2">
-        <v>1.7080428500000004</v>
+        <v>1.2080171000000002</v>
       </c>
       <c r="C97" s="2">
-        <v>2.6178458</v>
+        <v>3.1227498499999999</v>
       </c>
       <c r="D97" s="3"/>
     </row>
-    <row r="98" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B98" s="2">
-        <v>1.9999278000000005</v>
+        <v>1.0535376000000001</v>
       </c>
       <c r="C98" s="2">
-        <v>2.2544124500000002</v>
+        <v>3.0861625999999998</v>
       </c>
       <c r="D98" s="3"/>
     </row>
     <row r="99" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B99" s="2">
-        <v>2.1812379500000008</v>
+        <v>1.9153706000000001</v>
       </c>
       <c r="C99" s="2">
-        <v>2.8983480500000005</v>
+        <v>2.6828897999999999</v>
       </c>
       <c r="D99" s="3"/>
     </row>
     <row r="100" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B100" s="2">
-        <v>-0.27335999999999994</v>
+        <v>1.9235011000000002</v>
       </c>
       <c r="C100" s="2">
-        <v>1.3665618500000005</v>
+        <v>2.4454792000000003</v>
       </c>
       <c r="D100" s="3"/>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B101" s="2">
-        <v>-0.25709899999999986</v>
+        <v>1.3722531999999998</v>
       </c>
       <c r="C101" s="2">
-        <v>1.3177788500000003</v>
+        <v>2.2031903000000002</v>
       </c>
       <c r="D101" s="3"/>
     </row>
     <row r="102" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B102" s="2">
-        <v>-0.2749860999999999</v>
+        <v>1.5934028000000002</v>
       </c>
       <c r="C102" s="2">
-        <v>1.2584262000000002</v>
+        <v>2.3300261000000004</v>
       </c>
       <c r="D102" s="3"/>
     </row>
     <row r="103" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B103" s="2">
-        <v>-0.30750809999999995</v>
+        <v>1.1380948000000002</v>
       </c>
       <c r="C103" s="2">
-        <v>0.10308215000000009</v>
+        <v>2.2113207999999998</v>
       </c>
       <c r="D103" s="3"/>
     </row>
@@ -2366,106 +2306,98 @@
         <v>97</v>
       </c>
       <c r="B104" s="2">
-        <v>-0.26279034999999984</v>
-      </c>
-      <c r="C104" s="2">
-        <v>1.2909482000000003</v>
-      </c>
-      <c r="D104" s="3"/>
+        <v>1.5299849000000001</v>
+      </c>
+      <c r="C104" s="1">
+        <v>2.1901815</v>
+      </c>
     </row>
     <row r="105" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B105" s="2">
-        <v>1.385262</v>
-      </c>
-      <c r="C105" s="2">
-        <v>2.4227137999999999</v>
-      </c>
-      <c r="D105" s="3"/>
+        <v>1.6129160000000002</v>
+      </c>
+      <c r="C105" s="1">
+        <v>1.8291873000000005</v>
+      </c>
     </row>
     <row r="106" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B106" s="2">
-        <v>1.1315904000000003</v>
-      </c>
-      <c r="C106" s="2">
-        <v>2.4145833000000003</v>
-      </c>
-      <c r="D106" s="3"/>
+        <v>1.5364893000000004</v>
+      </c>
+      <c r="C106" s="1">
+        <v>2.1576595000000003</v>
+      </c>
     </row>
     <row r="107" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>100</v>
       </c>
       <c r="B107" s="2">
-        <v>1.2080171000000002</v>
-      </c>
-      <c r="C107" s="2">
-        <v>3.1227498499999999</v>
-      </c>
-      <c r="D107" s="3"/>
-    </row>
-    <row r="108" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>2.7739514000000005</v>
+      </c>
+      <c r="C107" s="1">
+        <v>2.2552255000000003</v>
+      </c>
+    </row>
+    <row r="108" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>101</v>
       </c>
       <c r="B108" s="2">
-        <v>1.0535376000000001</v>
-      </c>
-      <c r="C108" s="2">
-        <v>3.0861625999999998</v>
-      </c>
-      <c r="D108" s="3"/>
+        <v>1.4446146500000001</v>
+      </c>
+      <c r="C108" s="1">
+        <v>2.2292079</v>
+      </c>
     </row>
     <row r="109" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>102</v>
       </c>
       <c r="B109" s="2">
-        <v>1.9153706000000001</v>
-      </c>
-      <c r="C109" s="2">
-        <v>2.6828897999999999</v>
-      </c>
-      <c r="D109" s="3"/>
+        <v>1.6714556000000003</v>
+      </c>
+      <c r="C109" s="1">
+        <v>2.3690525000000004</v>
+      </c>
     </row>
     <row r="110" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>103</v>
       </c>
       <c r="B110" s="2">
-        <v>1.9235011000000002</v>
-      </c>
-      <c r="C110" s="2">
-        <v>2.4454792000000003</v>
-      </c>
-      <c r="D110" s="3"/>
+        <v>1.1055728</v>
+      </c>
+      <c r="C110" s="1">
+        <v>3.2422681999999998</v>
+      </c>
     </row>
     <row r="111" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>104</v>
       </c>
       <c r="B111" s="2">
-        <v>1.3722531999999998</v>
-      </c>
-      <c r="C111" s="2">
-        <v>2.2031903000000002</v>
-      </c>
-      <c r="D111" s="3"/>
+        <v>0.93971060000000017</v>
+      </c>
+      <c r="C111" s="1">
+        <v>2.5739411000000003</v>
+      </c>
     </row>
     <row r="112" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B112" s="2">
-        <v>1.5934028000000002</v>
+        <v>1.22996945</v>
       </c>
       <c r="C112" s="2">
-        <v>2.3300261000000004</v>
+        <v>2.5471104500000004</v>
       </c>
       <c r="D112" s="3"/>
     </row>
@@ -2474,22 +2406,21 @@
         <v>106</v>
       </c>
       <c r="B113" s="2">
-        <v>1.1380948000000002</v>
-      </c>
-      <c r="C113" s="2">
-        <v>2.2113207999999998</v>
-      </c>
-      <c r="D113" s="3"/>
+        <v>1.4356711000000004</v>
+      </c>
+      <c r="C113" s="1">
+        <v>1.8552049000000004</v>
+      </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>107</v>
       </c>
       <c r="B114" s="2">
-        <v>1.5299849000000001</v>
+        <v>1.3885141999999999</v>
       </c>
       <c r="C114" s="1">
-        <v>2.1901815</v>
+        <v>2.0861111000000001</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.35">
@@ -2497,10 +2428,10 @@
         <v>108</v>
       </c>
       <c r="B115" s="2">
-        <v>1.6129160000000002</v>
+        <v>1.4974628999999999</v>
       </c>
       <c r="C115" s="1">
-        <v>1.8291873000000005</v>
+        <v>2.2373384000000005</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.35">
@@ -2508,21 +2439,21 @@
         <v>109</v>
       </c>
       <c r="B116" s="2">
-        <v>1.5364893000000004</v>
+        <v>2.6251632500000004</v>
       </c>
       <c r="C116" s="1">
-        <v>2.1576595000000003</v>
-      </c>
-    </row>
-    <row r="117" spans="1:4" x14ac:dyDescent="0.35">
+        <v>2.5219058999999997</v>
+      </c>
+    </row>
+    <row r="117" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>110</v>
       </c>
       <c r="B117" s="2">
-        <v>2.7739514000000005</v>
+        <v>1.4893323999999999</v>
       </c>
       <c r="C117" s="1">
-        <v>2.2552255000000003</v>
+        <v>3.0910409000000003</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.35">
@@ -2530,10 +2461,10 @@
         <v>111</v>
       </c>
       <c r="B118" s="2">
-        <v>1.4446146500000001</v>
+        <v>1.0275200000000007</v>
       </c>
       <c r="C118" s="1">
-        <v>2.2292079</v>
+        <v>3.0455101</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.35">
@@ -2541,10 +2472,10 @@
         <v>112</v>
       </c>
       <c r="B119" s="2">
-        <v>1.6714556000000003</v>
+        <v>0.75270910000000057</v>
       </c>
       <c r="C119" s="1">
-        <v>2.3690525000000004</v>
+        <v>2.3462871000000001</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.35">
@@ -2552,10 +2483,10 @@
         <v>113</v>
       </c>
       <c r="B120" s="2">
-        <v>1.1055728</v>
+        <v>1.4015230000000001</v>
       </c>
       <c r="C120" s="1">
-        <v>3.2422681999999998</v>
+        <v>2.3218956000000004</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.35">
@@ -2563,33 +2494,33 @@
         <v>114</v>
       </c>
       <c r="B121" s="2">
-        <v>0.93971060000000017</v>
-      </c>
-      <c r="C121" s="1">
-        <v>2.5739411000000003</v>
-      </c>
+        <v>1.4421755000000003</v>
+      </c>
+      <c r="C121" s="2">
+        <v>1.8893530000000003</v>
+      </c>
+      <c r="D121" s="3"/>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A122" s="1" t="s">
         <v>115</v>
       </c>
       <c r="B122" s="2">
-        <v>1.22996945</v>
-      </c>
-      <c r="C122" s="2">
-        <v>2.5471104500000004</v>
-      </c>
-      <c r="D122" s="3"/>
+        <v>1.8982965500000004</v>
+      </c>
+      <c r="C122" s="1">
+        <v>2.5227189499999998</v>
+      </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A123" s="1" t="s">
         <v>116</v>
       </c>
       <c r="B123" s="2">
-        <v>1.4356711000000004</v>
+        <v>1.4494929500000002</v>
       </c>
       <c r="C123" s="1">
-        <v>1.8552049000000004</v>
+        <v>1.9226880499999996</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.35">
@@ -2597,10 +2528,10 @@
         <v>117</v>
       </c>
       <c r="B124" s="2">
-        <v>1.3885141999999999</v>
+        <v>2.1332680000000006</v>
       </c>
       <c r="C124" s="1">
-        <v>2.0861111000000001</v>
+        <v>2.3853135000000001</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.35">
@@ -2608,10 +2539,10 @@
         <v>118</v>
       </c>
       <c r="B125" s="2">
-        <v>1.4974628999999999</v>
+        <v>3.3024339000000005</v>
       </c>
       <c r="C125" s="1">
-        <v>2.2373384000000005</v>
+        <v>0.42748910000000029</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.35">
@@ -2619,21 +2550,21 @@
         <v>119</v>
       </c>
       <c r="B126" s="2">
-        <v>2.6251632500000004</v>
+        <v>4.7106365000000006</v>
       </c>
       <c r="C126" s="1">
-        <v>2.5219058999999997</v>
-      </c>
-    </row>
-    <row r="127" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0.39008880000000024</v>
+      </c>
+    </row>
+    <row r="127" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A127" s="1" t="s">
         <v>120</v>
       </c>
       <c r="B127" s="2">
-        <v>1.4893323999999999</v>
+        <v>4.4976174000000002</v>
       </c>
       <c r="C127" s="1">
-        <v>3.0910409000000003</v>
+        <v>0.36244510000000019</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.35">
@@ -2641,10 +2572,10 @@
         <v>121</v>
       </c>
       <c r="B128" s="2">
-        <v>1.0275200000000007</v>
+        <v>3.7471722500000002</v>
       </c>
       <c r="C128" s="1">
-        <v>3.0455101</v>
+        <v>0.47871124999999992</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.35">
@@ -2652,10 +2583,10 @@
         <v>122</v>
       </c>
       <c r="B129" s="2">
-        <v>0.75270910000000057</v>
+        <v>1.5714504500000004</v>
       </c>
       <c r="C129" s="1">
-        <v>2.3462871000000001</v>
+        <v>0.39821930000000028</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.35">
@@ -2663,10 +2594,10 @@
         <v>123</v>
       </c>
       <c r="B130" s="2">
-        <v>1.4015230000000001</v>
+        <v>1.5129108500000004</v>
       </c>
       <c r="C130" s="1">
-        <v>2.3218956000000004</v>
+        <v>0.28357925000000006</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.35">
@@ -2674,22 +2605,21 @@
         <v>124</v>
       </c>
       <c r="B131" s="2">
-        <v>1.4421755000000003</v>
-      </c>
-      <c r="C131" s="2">
-        <v>1.8893530000000003</v>
-      </c>
-      <c r="D131" s="3"/>
+        <v>2.0747283999999997</v>
+      </c>
+      <c r="C131" s="1">
+        <v>0.26813130000000007</v>
+      </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A132" s="1" t="s">
         <v>125</v>
       </c>
       <c r="B132" s="2">
-        <v>1.8982965500000004</v>
+        <v>1.8064219000000001</v>
       </c>
       <c r="C132" s="1">
-        <v>2.5227189499999998</v>
+        <v>0.36081900000000022</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.35">
@@ -2697,10 +2627,10 @@
         <v>126</v>
       </c>
       <c r="B133" s="2">
-        <v>1.4494929500000002</v>
+        <v>4.3398857</v>
       </c>
       <c r="C133" s="1">
-        <v>1.9226880499999996</v>
+        <v>0.28601840000000012</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.35">
@@ -2708,120 +2638,120 @@
         <v>127</v>
       </c>
       <c r="B134" s="2">
-        <v>2.1332680000000006</v>
+        <v>4.1935366999999992</v>
       </c>
       <c r="C134" s="1">
-        <v>2.3853135000000001</v>
-      </c>
-    </row>
-    <row r="135" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.66164750000000017</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A135" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B135" s="2">
-        <v>3.3024339000000005</v>
+        <v>3.6325322</v>
       </c>
       <c r="C135" s="1">
-        <v>0.42748910000000029</v>
-      </c>
-    </row>
-    <row r="136" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.44862840000000004</v>
+      </c>
+    </row>
+    <row r="136" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A136" s="1" t="s">
         <v>129</v>
       </c>
       <c r="B136" s="2">
-        <v>4.7106365000000006</v>
+        <v>5.3627026000000004</v>
       </c>
       <c r="C136" s="1">
-        <v>0.39008880000000024</v>
-      </c>
-    </row>
-    <row r="137" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.16650005000000001</v>
+      </c>
+    </row>
+    <row r="137" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A137" s="1" t="s">
         <v>130</v>
       </c>
       <c r="B137" s="2">
-        <v>4.4976174000000002</v>
+        <v>3.8276642000000001</v>
       </c>
       <c r="C137" s="1">
-        <v>0.36244510000000019</v>
-      </c>
-    </row>
-    <row r="138" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.16406090000000018</v>
+      </c>
+    </row>
+    <row r="138" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A138" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B138" s="2">
-        <v>3.7471722500000002</v>
+        <v>3.5764317500000011</v>
       </c>
       <c r="C138" s="1">
-        <v>0.47871124999999992</v>
-      </c>
-    </row>
-    <row r="139" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.12991280000000005</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A139" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B139" s="2">
-        <v>1.5714504500000004</v>
+        <v>6.2554315000000003</v>
       </c>
       <c r="C139" s="1">
-        <v>0.39821930000000028</v>
-      </c>
-    </row>
-    <row r="140" spans="1:4" x14ac:dyDescent="0.35">
+        <v>8.8447250000000199E-2</v>
+      </c>
+    </row>
+    <row r="140" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A140" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B140" s="2">
-        <v>1.5129108500000004</v>
+        <v>4.5155045000000005</v>
       </c>
       <c r="C140" s="1">
-        <v>0.28357925000000006</v>
-      </c>
-    </row>
-    <row r="141" spans="1:4" x14ac:dyDescent="0.35">
+        <v>9.5764700000000147E-2</v>
+      </c>
+    </row>
+    <row r="141" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A141" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B141" s="2">
-        <v>2.0747283999999997</v>
+        <v>5.7464622000000016</v>
       </c>
       <c r="C141" s="1">
-        <v>0.26813130000000007</v>
-      </c>
-    </row>
-    <row r="142" spans="1:4" x14ac:dyDescent="0.35">
+        <v>6.1616600000000132E-2</v>
+      </c>
+    </row>
+    <row r="142" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A142" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B142" s="2">
-        <v>1.8064219000000001</v>
+        <v>5.8082540000000007</v>
       </c>
       <c r="C142" s="1">
-        <v>0.36081900000000022</v>
-      </c>
-    </row>
-    <row r="143" spans="1:4" x14ac:dyDescent="0.35">
+        <v>0.14129550000000024</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A143" s="1" t="s">
         <v>136</v>
       </c>
       <c r="B143" s="2">
-        <v>4.3398857</v>
+        <v>3.1772241999999995</v>
       </c>
       <c r="C143" s="1">
-        <v>0.28601840000000012</v>
-      </c>
-    </row>
-    <row r="144" spans="1:4" x14ac:dyDescent="0.35">
+        <v>5.5112200000000056E-2</v>
+      </c>
+    </row>
+    <row r="144" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A144" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B144" s="2">
-        <v>4.1935366999999992</v>
+        <v>2.3966962000000001</v>
       </c>
       <c r="C144" s="1">
-        <v>0.66164750000000017</v>
+        <v>8.4382000000000179E-2</v>
       </c>
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.35">
@@ -2829,10 +2759,10 @@
         <v>138</v>
       </c>
       <c r="B145" s="2">
-        <v>3.6325322</v>
+        <v>5.7968713000000003</v>
       </c>
       <c r="C145" s="1">
-        <v>0.44862840000000004</v>
+        <v>0.12178230000000023</v>
       </c>
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.35">
@@ -2840,10 +2770,10 @@
         <v>139</v>
       </c>
       <c r="B146" s="2">
-        <v>5.3627026000000004</v>
+        <v>7.9351928000000012</v>
       </c>
       <c r="C146" s="1">
-        <v>0.16650005000000001</v>
+        <v>6.812100000000032E-2</v>
       </c>
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.35">
@@ -2851,10 +2781,10 @@
         <v>140</v>
       </c>
       <c r="B147" s="2">
-        <v>3.8276642000000001</v>
+        <v>8.400257400000001</v>
       </c>
       <c r="C147" s="1">
-        <v>0.16406090000000018</v>
+        <v>0.10552130000000015</v>
       </c>
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.35">
@@ -2862,10 +2792,10 @@
         <v>141</v>
       </c>
       <c r="B148" s="2">
-        <v>3.5764317500000011</v>
+        <v>8.7986518999999994</v>
       </c>
       <c r="C148" s="1">
-        <v>0.12991280000000005</v>
+        <v>0.12503450000000016</v>
       </c>
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.35">
@@ -2873,10 +2803,10 @@
         <v>142</v>
       </c>
       <c r="B149" s="2">
-        <v>6.2554315000000003</v>
+        <v>1.8690267500000002</v>
       </c>
       <c r="C149" s="1">
-        <v>8.8447250000000199E-2</v>
+        <v>2.5842400000000154E-2</v>
       </c>
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.35">
@@ -2884,10 +2814,10 @@
         <v>143</v>
       </c>
       <c r="B150" s="2">
-        <v>4.5155045000000005</v>
+        <v>2.5739411000000003</v>
       </c>
       <c r="C150" s="1">
-        <v>9.5764700000000147E-2</v>
+        <v>0.10064300000000004</v>
       </c>
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.35">
@@ -2895,10 +2825,10 @@
         <v>144</v>
       </c>
       <c r="B151" s="2">
-        <v>5.7464622000000016</v>
+        <v>4.5252611000000007</v>
       </c>
       <c r="C151" s="1">
-        <v>6.1616600000000132E-2</v>
+        <v>9.0886400000000034E-2</v>
       </c>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.35">
@@ -2906,21 +2836,21 @@
         <v>145</v>
       </c>
       <c r="B152" s="2">
-        <v>5.8082540000000007</v>
+        <v>5.7903668999999995</v>
       </c>
       <c r="C152" s="1">
-        <v>0.14129550000000024</v>
-      </c>
-    </row>
-    <row r="153" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0.11039960000000004</v>
+      </c>
+    </row>
+    <row r="153" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A153" s="1" t="s">
         <v>146</v>
       </c>
       <c r="B153" s="2">
-        <v>3.1772241999999995</v>
+        <v>4.5106261999999999</v>
       </c>
       <c r="C153" s="1">
-        <v>5.5112200000000056E-2</v>
+        <v>6.3242700000000096E-2</v>
       </c>
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.35">
@@ -2928,10 +2858,10 @@
         <v>147</v>
       </c>
       <c r="B154" s="2">
-        <v>2.3966962000000001</v>
+        <v>5.5643390000000004</v>
       </c>
       <c r="C154" s="1">
-        <v>8.4382000000000179E-2</v>
+        <v>0.12666060000000012</v>
       </c>
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.35">
@@ -2939,10 +2869,10 @@
         <v>148</v>
       </c>
       <c r="B155" s="2">
-        <v>5.7968713000000003</v>
+        <v>-0.26848169999999993</v>
       </c>
       <c r="C155" s="1">
-        <v>0.12178230000000023</v>
+        <v>-0.15790689999999985</v>
       </c>
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.35">
@@ -2950,10 +2880,10 @@
         <v>149</v>
       </c>
       <c r="B156" s="2">
-        <v>7.9351928000000012</v>
+        <v>-0.25222069999999985</v>
       </c>
       <c r="C156" s="1">
-        <v>6.812100000000032E-2</v>
+        <v>-0.12863709999999984</v>
       </c>
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.35">
@@ -2961,10 +2891,10 @@
         <v>150</v>
       </c>
       <c r="B157" s="2">
-        <v>8.400257400000001</v>
+        <v>0.74701775000000037</v>
       </c>
       <c r="C157" s="1">
-        <v>0.10552130000000015</v>
+        <v>0.56895980000000002</v>
       </c>
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.35">
@@ -2972,10 +2902,10 @@
         <v>151</v>
       </c>
       <c r="B158" s="2">
-        <v>8.7986518999999994</v>
+        <v>0.63725600000000027</v>
       </c>
       <c r="C158" s="1">
-        <v>0.12503450000000016</v>
+        <v>0.47952430000000024</v>
       </c>
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.35">
@@ -2983,120 +2913,120 @@
         <v>152</v>
       </c>
       <c r="B159" s="2">
-        <v>1.8690267500000002</v>
+        <v>0.55595099999999986</v>
       </c>
       <c r="C159" s="1">
-        <v>2.5842400000000154E-2</v>
+        <v>0.58684690000000028</v>
       </c>
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A160" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B160" s="2">
-        <v>2.5739411000000003</v>
+        <v>0.56895980000000002</v>
       </c>
       <c r="C160" s="1">
-        <v>0.10064300000000004</v>
+        <v>0.61774280000000026</v>
       </c>
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A161" s="1" t="s">
-        <v>154</v>
-      </c>
-      <c r="B161" s="2">
-        <v>4.5252611000000007</v>
+        <v>153</v>
+      </c>
+      <c r="B161" s="5">
+        <v>0.54944660000000001</v>
       </c>
       <c r="C161" s="1">
-        <v>9.0886400000000034E-2</v>
+        <v>0.71368270000000034</v>
       </c>
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A162" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B162" s="2">
-        <v>5.7903668999999995</v>
+        <v>-0.18880280000000005</v>
       </c>
       <c r="C162" s="1">
-        <v>0.11039960000000004</v>
+        <v>1.2372869000000004</v>
       </c>
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A163" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B163" s="2">
-        <v>4.5106261999999999</v>
+        <v>-0.17579400000000001</v>
       </c>
       <c r="C163" s="1">
-        <v>6.3242700000000096E-2</v>
+        <v>1.1445992</v>
       </c>
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A164" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B164" s="2">
-        <v>5.5643390000000004</v>
+        <v>0.58034250000000021</v>
       </c>
       <c r="C164" s="1">
-        <v>0.12666060000000012</v>
+        <v>0.58603385000000019</v>
       </c>
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A165" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B165" s="2">
-        <v>-0.26848169999999993</v>
+        <v>0.52505510000000011</v>
       </c>
       <c r="C165" s="1">
-        <v>-0.15790689999999985</v>
+        <v>0.32748395000000019</v>
       </c>
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A166" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B166" s="2">
-        <v>-0.25222069999999985</v>
+        <v>-1.9688399999999828E-2</v>
       </c>
       <c r="C166" s="1">
-        <v>-0.12863709999999984</v>
+        <v>1.5446198000000004</v>
       </c>
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A167" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="B167" s="2">
+        <v>-8.3056999999999714E-3</v>
+      </c>
+      <c r="C167" s="1">
+        <v>1.2641175500000004</v>
+      </c>
+    </row>
+    <row r="168" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A168" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="B167" s="2">
-        <v>0.74701775000000037</v>
-      </c>
-      <c r="C167" s="1">
-        <v>0.56895980000000002</v>
-      </c>
-    </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A168" s="1" t="s">
-        <v>161</v>
-      </c>
       <c r="B168" s="2">
-        <v>0.63725600000000027</v>
+        <v>0.62262110000000015</v>
       </c>
       <c r="C168" s="1">
-        <v>0.47952430000000024</v>
+        <v>0.94946720000000018</v>
       </c>
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A169" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B169" s="2">
-        <v>0.55595099999999986</v>
+        <v>0.26894435000000017</v>
       </c>
       <c r="C169" s="1">
-        <v>0.58684690000000028</v>
+        <v>0.80311820000000012</v>
       </c>
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.35">
@@ -3104,21 +3034,21 @@
         <v>162</v>
       </c>
       <c r="B170" s="2">
-        <v>0.56895980000000002</v>
+        <v>0.37708000000000008</v>
       </c>
       <c r="C170" s="1">
-        <v>0.61774280000000026</v>
+        <v>0.51285935000000005</v>
       </c>
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A171" s="1" t="s">
         <v>163</v>
       </c>
-      <c r="B171" s="5">
-        <v>0.54944660000000001</v>
+      <c r="B171" s="2">
+        <v>0.33317530000000017</v>
       </c>
       <c r="C171" s="1">
-        <v>0.71368270000000034</v>
+        <v>0.53318559999999993</v>
       </c>
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.35">
@@ -3126,10 +3056,10 @@
         <v>164</v>
       </c>
       <c r="B172" s="2">
-        <v>-0.18880280000000005</v>
+        <v>0.16080870000000025</v>
       </c>
       <c r="C172" s="1">
-        <v>1.2372869000000004</v>
+        <v>1.0494723500000001</v>
       </c>
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.35">
@@ -3137,10 +3067,10 @@
         <v>165</v>
       </c>
       <c r="B173" s="2">
-        <v>-0.17579400000000001</v>
+        <v>9.0886400000000034E-2</v>
       </c>
       <c r="C173" s="1">
-        <v>1.1445992</v>
+        <v>0.85190120000000014</v>
       </c>
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.35">
@@ -3148,10 +3078,10 @@
         <v>166</v>
       </c>
       <c r="B174" s="2">
-        <v>0.58034250000000021</v>
+        <v>-0.21644649999999988</v>
       </c>
       <c r="C174" s="1">
-        <v>0.58603385000000019</v>
+        <v>1.6161682000000006</v>
       </c>
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.35">
@@ -3159,10 +3089,10 @@
         <v>167</v>
       </c>
       <c r="B175" s="2">
-        <v>0.52505510000000011</v>
+        <v>-0.23595969999999988</v>
       </c>
       <c r="C175" s="1">
-        <v>0.32748395000000019</v>
+        <v>1.4543712500000003</v>
       </c>
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.35">
@@ -3170,10 +3100,10 @@
         <v>168</v>
       </c>
       <c r="B176" s="2">
-        <v>-1.9688399999999828E-2</v>
+        <v>0.13966940000000005</v>
       </c>
       <c r="C176" s="1">
-        <v>1.5446198000000004</v>
+        <v>1.0470332000000002</v>
       </c>
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.35">
@@ -3181,21 +3111,21 @@
         <v>169</v>
       </c>
       <c r="B177" s="2">
-        <v>-8.3056999999999714E-3</v>
+        <v>0.10552130000000015</v>
       </c>
       <c r="C177" s="1">
-        <v>1.2641175500000004</v>
-      </c>
-    </row>
-    <row r="178" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>1.0714247000000003</v>
+      </c>
+    </row>
+    <row r="178" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A178" s="1" t="s">
         <v>170</v>
       </c>
       <c r="B178" s="2">
-        <v>0.62262110000000015</v>
+        <v>0.30065330000000023</v>
       </c>
       <c r="C178" s="1">
-        <v>0.94946720000000018</v>
+        <v>1.2055779500000003</v>
       </c>
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.35">
@@ -3203,10 +3133,10 @@
         <v>171</v>
       </c>
       <c r="B179" s="2">
-        <v>0.26894435000000017</v>
+        <v>0.24861810000000006</v>
       </c>
       <c r="C179" s="1">
-        <v>0.80311820000000012</v>
+        <v>1.2446043500000004</v>
       </c>
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.35">
@@ -3214,10 +3144,10 @@
         <v>172</v>
       </c>
       <c r="B180" s="2">
-        <v>0.37708000000000008</v>
+        <v>0.46163719999999997</v>
       </c>
       <c r="C180" s="1">
-        <v>0.51285935000000005</v>
+        <v>1.8251220500000001</v>
       </c>
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.35">
@@ -3225,10 +3155,10 @@
         <v>173</v>
       </c>
       <c r="B181" s="2">
-        <v>0.33317530000000017</v>
+        <v>0.30797075000000018</v>
       </c>
       <c r="C181" s="1">
-        <v>0.53318559999999993</v>
+        <v>1.5381153999999997</v>
       </c>
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.35">
@@ -3236,10 +3166,10 @@
         <v>174</v>
       </c>
       <c r="B182" s="2">
-        <v>0.16080870000000025</v>
+        <v>-0.15302859999999985</v>
       </c>
       <c r="C182" s="1">
-        <v>1.0494723500000001</v>
+        <v>0.8738535500000002</v>
       </c>
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.35">
@@ -3247,120 +3177,120 @@
         <v>175</v>
       </c>
       <c r="B183" s="2">
-        <v>9.0886400000000034E-2</v>
+        <v>0.11039960000000026</v>
       </c>
       <c r="C183" s="1">
-        <v>0.85190120000000014</v>
+        <v>0.75433520000000009</v>
       </c>
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A184" s="1" t="s">
+      <c r="A184" t="s">
         <v>176</v>
       </c>
-      <c r="B184" s="2">
-        <v>-0.21644649999999988</v>
-      </c>
-      <c r="C184" s="1">
-        <v>1.6161682000000006</v>
+      <c r="B184" s="6">
+        <v>0.58118133333333333</v>
+      </c>
+      <c r="C184" s="7">
+        <v>1.3682519333333329</v>
       </c>
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A185" s="1" t="s">
+      <c r="A185" t="s">
         <v>177</v>
       </c>
-      <c r="B185" s="2">
-        <v>-0.23595969999999988</v>
-      </c>
-      <c r="C185" s="1">
-        <v>1.4543712500000003</v>
+      <c r="B185" s="6">
+        <v>0.31574766666666665</v>
+      </c>
+      <c r="C185" s="7">
+        <v>1.4952154666666668</v>
       </c>
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A186" s="1" t="s">
+      <c r="A186" t="s">
         <v>178</v>
       </c>
-      <c r="B186" s="2">
-        <v>0.13966940000000005</v>
-      </c>
-      <c r="C186" s="1">
-        <v>1.0470332000000002</v>
+      <c r="B186" s="6">
+        <v>0.31794133333333352</v>
+      </c>
+      <c r="C186" s="7">
+        <v>1.4646799333333334</v>
       </c>
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A187" s="1" t="s">
+      <c r="A187" t="s">
         <v>179</v>
       </c>
-      <c r="B187" s="2">
-        <v>0.10552130000000015</v>
-      </c>
-      <c r="C187" s="1">
-        <v>1.0714247000000003</v>
+      <c r="B187" s="6">
+        <v>0.62066733333333346</v>
+      </c>
+      <c r="C187" s="7">
+        <v>1.4068231333333332</v>
       </c>
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A188" s="1" t="s">
+      <c r="A188" t="s">
         <v>180</v>
       </c>
-      <c r="B188" s="2">
-        <v>0.30065330000000023</v>
-      </c>
-      <c r="C188" s="1">
-        <v>1.2055779500000003</v>
+      <c r="B188" s="6">
+        <v>-8.9150000000000063E-3</v>
+      </c>
+      <c r="C188" s="7">
+        <v>0.1098665333333334</v>
       </c>
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A189" s="1" t="s">
+      <c r="A189" t="s">
         <v>181</v>
       </c>
-      <c r="B189" s="2">
-        <v>0.24861810000000006</v>
-      </c>
-      <c r="C189" s="1">
-        <v>1.2446043500000004</v>
+      <c r="B189" s="6">
+        <v>-1.3302333333333305E-2</v>
+      </c>
+      <c r="C189" s="7">
+        <v>5.3616866666666541E-2</v>
       </c>
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A190" s="1" t="s">
+      <c r="A190" t="s">
         <v>182</v>
       </c>
-      <c r="B190" s="2">
-        <v>0.46163719999999997</v>
-      </c>
-      <c r="C190" s="1">
-        <v>1.8251220500000001</v>
+      <c r="B190" s="6">
+        <v>-2.8657999999999961E-2</v>
+      </c>
+      <c r="C190" s="7">
+        <v>8.7366666666666593E-2</v>
       </c>
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A191" s="1" t="s">
+      <c r="A191" t="s">
         <v>183</v>
       </c>
-      <c r="B191" s="2">
-        <v>0.30797075000000018</v>
-      </c>
-      <c r="C191" s="1">
-        <v>1.5381153999999997</v>
+      <c r="B191" s="6">
+        <v>3.3934620000000004</v>
+      </c>
+      <c r="C191" s="7">
+        <v>0.19263390000000002</v>
       </c>
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A192" s="1" t="s">
+      <c r="A192" t="s">
         <v>184</v>
       </c>
-      <c r="B192" s="2">
-        <v>-0.15302859999999985</v>
-      </c>
-      <c r="C192" s="1">
-        <v>0.8738535500000002</v>
+      <c r="B192" s="6">
+        <v>3.8958116666666669</v>
+      </c>
+      <c r="C192" s="7">
+        <v>0.22397299999999987</v>
       </c>
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A193" s="1" t="s">
+      <c r="A193" t="s">
         <v>185</v>
       </c>
-      <c r="B193" s="2">
-        <v>0.11039960000000026</v>
-      </c>
-      <c r="C193" s="1">
-        <v>0.75433520000000009</v>
+      <c r="B193" s="6">
+        <v>5.661713333333334</v>
+      </c>
+      <c r="C193" s="7">
+        <v>0.29790113333333346</v>
       </c>
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.35">
@@ -3368,10 +3298,10 @@
         <v>186</v>
       </c>
       <c r="B194" s="6">
-        <v>0.58118133333333333</v>
+        <v>5.2449166666666676</v>
       </c>
       <c r="C194" s="7">
-        <v>1.3682519333333329</v>
+        <v>1.8259933333333311E-2</v>
       </c>
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.35">
@@ -3379,10 +3309,10 @@
         <v>187</v>
       </c>
       <c r="B195" s="6">
-        <v>0.31574766666666665</v>
+        <v>4.6986936666666663</v>
       </c>
       <c r="C195" s="7">
-        <v>1.4952154666666668</v>
+        <v>6.2456100000000014E-2</v>
       </c>
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.35">
@@ -3390,10 +3320,10 @@
         <v>188</v>
       </c>
       <c r="B196" s="6">
-        <v>0.31794133333333352</v>
+        <v>4.7315986666666676</v>
       </c>
       <c r="C196" s="7">
-        <v>1.4646799333333334</v>
+        <v>0.22718726666666655</v>
       </c>
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.35">
@@ -3401,21 +3331,21 @@
         <v>189</v>
       </c>
       <c r="B197" s="6">
-        <v>0.62066733333333346</v>
+        <v>3.2596483333333337</v>
       </c>
       <c r="C197" s="7">
-        <v>1.4068231333333332</v>
-      </c>
-    </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.35">
+        <v>0.20468739999999985</v>
+      </c>
+    </row>
+    <row r="198" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A198" t="s">
         <v>190</v>
       </c>
       <c r="B198" s="6">
-        <v>-8.9150000000000063E-3</v>
+        <v>2.0114520000000002</v>
       </c>
       <c r="C198" s="7">
-        <v>0.1098665333333334</v>
+        <v>0.20790166666666654</v>
       </c>
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.35">
@@ -3423,10 +3353,10 @@
         <v>191</v>
       </c>
       <c r="B199" s="6">
-        <v>-1.3302333333333305E-2</v>
+        <v>3.44611</v>
       </c>
       <c r="C199" s="7">
-        <v>5.3616866666666541E-2</v>
+        <v>0.23120510000000005</v>
       </c>
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.35">
@@ -3434,10 +3364,10 @@
         <v>192</v>
       </c>
       <c r="B200" s="6">
-        <v>-2.8657999999999961E-2</v>
+        <v>3.9374913333333339</v>
       </c>
       <c r="C200" s="7">
-        <v>8.7366666666666593E-2</v>
+        <v>0.22638370000000008</v>
       </c>
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.35">
@@ -3445,10 +3375,10 @@
         <v>193</v>
       </c>
       <c r="B201" s="6">
-        <v>3.3934620000000004</v>
+        <v>6.9472019999999999</v>
       </c>
       <c r="C201" s="7">
-        <v>0.19263390000000002</v>
+        <v>0.26575846666666658</v>
       </c>
     </row>
     <row r="202" spans="1:3" x14ac:dyDescent="0.35">
@@ -3456,10 +3386,10 @@
         <v>194</v>
       </c>
       <c r="B202" s="6">
-        <v>3.8958116666666669</v>
+        <v>6.8901666666666683</v>
       </c>
       <c r="C202" s="7">
-        <v>0.22397299999999987</v>
+        <v>0.20790166666666654</v>
       </c>
     </row>
     <row r="203" spans="1:3" x14ac:dyDescent="0.35">
@@ -3467,10 +3397,10 @@
         <v>195</v>
       </c>
       <c r="B203" s="6">
-        <v>5.661713333333334</v>
+        <v>4.768891</v>
       </c>
       <c r="C203" s="7">
-        <v>0.29790113333333346</v>
+        <v>0.20468739999999996</v>
       </c>
     </row>
     <row r="204" spans="1:3" x14ac:dyDescent="0.35">
@@ -3478,10 +3408,10 @@
         <v>196</v>
       </c>
       <c r="B204" s="6">
-        <v>5.2449166666666676</v>
+        <v>4.1733105000000004</v>
       </c>
       <c r="C204" s="7">
-        <v>1.8259933333333311E-2</v>
+        <v>0.28182979999999991</v>
       </c>
     </row>
     <row r="205" spans="1:3" x14ac:dyDescent="0.35">
@@ -3489,10 +3419,10 @@
         <v>197</v>
       </c>
       <c r="B205" s="6">
-        <v>4.6986936666666663</v>
+        <v>4.0285285000000002</v>
       </c>
       <c r="C205" s="7">
-        <v>6.2456100000000014E-2</v>
+        <v>0.27218699999999996</v>
       </c>
     </row>
     <row r="206" spans="1:3" x14ac:dyDescent="0.35">
@@ -3500,10 +3430,10 @@
         <v>198</v>
       </c>
       <c r="B206" s="6">
-        <v>4.7315986666666676</v>
+        <v>3.9594279999999999</v>
       </c>
       <c r="C206" s="7">
-        <v>0.22718726666666655</v>
+        <v>0.30915106666666659</v>
       </c>
     </row>
     <row r="207" spans="1:3" x14ac:dyDescent="0.35">
@@ -3511,21 +3441,21 @@
         <v>199</v>
       </c>
       <c r="B207" s="6">
-        <v>3.2596483333333337</v>
+        <v>7.0261740000000001</v>
       </c>
       <c r="C207" s="7">
-        <v>0.20468739999999985</v>
-      </c>
-    </row>
-    <row r="208" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>0.70450586666666637</v>
+      </c>
+    </row>
+    <row r="208" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A208" t="s">
         <v>200</v>
       </c>
       <c r="B208" s="6">
-        <v>2.0114520000000002</v>
+        <v>13.9441132</v>
       </c>
       <c r="C208" s="7">
-        <v>0.20790166666666654</v>
+        <v>0.84420760000000006</v>
       </c>
     </row>
     <row r="209" spans="1:3" x14ac:dyDescent="0.35">
@@ -3533,10 +3463,10 @@
         <v>201</v>
       </c>
       <c r="B209" s="6">
-        <v>3.44611</v>
+        <v>4.3441696000000007</v>
       </c>
       <c r="C209" s="7">
-        <v>0.23120510000000005</v>
+        <v>0.31090993333333339</v>
       </c>
     </row>
     <row r="210" spans="1:3" x14ac:dyDescent="0.35">
@@ -3544,10 +3474,10 @@
         <v>202</v>
       </c>
       <c r="B210" s="6">
-        <v>3.9374913333333339</v>
+        <v>3.8769076000000005</v>
       </c>
       <c r="C210" s="7">
-        <v>0.22638370000000008</v>
+        <v>0.48920646666666667</v>
       </c>
     </row>
     <row r="211" spans="1:3" x14ac:dyDescent="0.35">
@@ -3555,10 +3485,10 @@
         <v>203</v>
       </c>
       <c r="B211" s="6">
-        <v>6.9472019999999999</v>
+        <v>4.2644602000000003</v>
       </c>
       <c r="C211" s="7">
-        <v>0.26575846666666658</v>
+        <v>0.31250186666666679</v>
       </c>
     </row>
     <row r="212" spans="1:3" x14ac:dyDescent="0.35">
@@ -3566,10 +3496,10 @@
         <v>204</v>
       </c>
       <c r="B212" s="6">
-        <v>6.8901666666666683</v>
+        <v>4.127946399999999</v>
       </c>
       <c r="C212" s="7">
-        <v>0.20790166666666654</v>
+        <v>0.66033929999999996</v>
       </c>
     </row>
     <row r="213" spans="1:3" x14ac:dyDescent="0.35">
@@ -3577,10 +3507,10 @@
         <v>205</v>
       </c>
       <c r="B213" s="6">
-        <v>4.768891</v>
+        <v>4.8444148000000009</v>
       </c>
       <c r="C213" s="7">
-        <v>0.20468739999999996</v>
+        <v>0.72242469999999992</v>
       </c>
     </row>
     <row r="214" spans="1:3" x14ac:dyDescent="0.35">
@@ -3588,10 +3518,10 @@
         <v>206</v>
       </c>
       <c r="B214" s="6">
-        <v>4.1733105000000004</v>
+        <v>6.1747372000000009</v>
       </c>
       <c r="C214" s="7">
-        <v>0.28182979999999991</v>
+        <v>0.73914000000000013</v>
       </c>
     </row>
     <row r="215" spans="1:3" x14ac:dyDescent="0.35">
@@ -3599,10 +3529,10 @@
         <v>207</v>
       </c>
       <c r="B215" s="6">
-        <v>4.0285285000000002</v>
+        <v>4.9232080000000007</v>
       </c>
       <c r="C215" s="7">
-        <v>0.27218699999999996</v>
+        <v>0.81316490000000008</v>
       </c>
     </row>
     <row r="216" spans="1:3" x14ac:dyDescent="0.35">
@@ -3610,274 +3540,54 @@
         <v>208</v>
       </c>
       <c r="B216" s="6">
-        <v>3.9594279999999999</v>
+        <v>3.5305840000000002</v>
       </c>
       <c r="C216" s="7">
-        <v>0.30915106666666659</v>
+        <v>0.66750300000000018</v>
       </c>
     </row>
     <row r="217" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A217" t="s">
         <v>209</v>
       </c>
-      <c r="B217" s="6">
-        <v>7.0261740000000001</v>
+      <c r="B217" s="7">
+        <v>6.4844127999999994</v>
       </c>
       <c r="C217" s="7">
-        <v>0.70450586666666637</v>
+        <v>0.65317560000000019</v>
       </c>
     </row>
     <row r="218" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A218" t="s">
         <v>210</v>
       </c>
-      <c r="B218" s="6">
-        <v>13.9441132</v>
+      <c r="B218" s="7">
+        <v>7.9539975999999992</v>
       </c>
       <c r="C218" s="7">
-        <v>0.84420760000000006</v>
+        <v>0.54333219999999982</v>
       </c>
     </row>
     <row r="219" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A219" t="s">
         <v>211</v>
       </c>
-      <c r="B219" s="6">
-        <v>4.3441696000000007</v>
+      <c r="B219" s="7">
+        <v>4.4046388000000007</v>
       </c>
       <c r="C219" s="7">
-        <v>0.31090993333333339</v>
+        <v>1.3042763333333331</v>
       </c>
     </row>
     <row r="220" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A220" t="s">
         <v>212</v>
       </c>
-      <c r="B220" s="6">
-        <v>3.8769076000000005</v>
+      <c r="B220" s="7">
+        <v>4.4321248000000004</v>
       </c>
       <c r="C220" s="7">
-        <v>0.48920646666666667</v>
-      </c>
-    </row>
-    <row r="221" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A221" t="s">
-        <v>213</v>
-      </c>
-      <c r="B221" s="6">
-        <v>4.2644602000000003</v>
-      </c>
-      <c r="C221" s="7">
-        <v>0.31250186666666679</v>
-      </c>
-    </row>
-    <row r="222" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A222" t="s">
-        <v>214</v>
-      </c>
-      <c r="B222" s="6">
-        <v>4.127946399999999</v>
-      </c>
-      <c r="C222" s="7">
-        <v>0.66033929999999996</v>
-      </c>
-    </row>
-    <row r="223" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A223" t="s">
-        <v>215</v>
-      </c>
-      <c r="B223" s="6">
-        <v>4.8444148000000009</v>
-      </c>
-      <c r="C223" s="7">
-        <v>0.72242469999999992</v>
-      </c>
-    </row>
-    <row r="224" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A224" t="s">
-        <v>216</v>
-      </c>
-      <c r="B224" s="6">
-        <v>6.1747372000000009</v>
-      </c>
-      <c r="C224" s="7">
-        <v>0.73914000000000013</v>
-      </c>
-    </row>
-    <row r="225" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A225" t="s">
-        <v>217</v>
-      </c>
-      <c r="B225" s="6">
-        <v>4.9232080000000007</v>
-      </c>
-      <c r="C225" s="7">
-        <v>0.81316490000000008</v>
-      </c>
-    </row>
-    <row r="226" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A226" t="s">
-        <v>218</v>
-      </c>
-      <c r="B226" s="6">
-        <v>3.5305840000000002</v>
-      </c>
-      <c r="C226" s="7">
-        <v>0.66750300000000018</v>
-      </c>
-    </row>
-    <row r="227" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A227" t="s">
-        <v>219</v>
-      </c>
-      <c r="B227" s="7">
-        <v>6.4844127999999994</v>
-      </c>
-      <c r="C227" s="7">
-        <v>0.65317560000000019</v>
-      </c>
-    </row>
-    <row r="228" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A228" t="s">
-        <v>220</v>
-      </c>
-      <c r="B228" s="7">
-        <v>7.9539975999999992</v>
-      </c>
-      <c r="C228" s="7">
-        <v>0.54333219999999982</v>
-      </c>
-    </row>
-    <row r="229" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A229" t="s">
-        <v>221</v>
-      </c>
-      <c r="B229" s="7">
-        <v>4.4046388000000007</v>
-      </c>
-      <c r="C229" s="7">
-        <v>1.3042763333333331</v>
-      </c>
-    </row>
-    <row r="230" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A230" t="s">
-        <v>222</v>
-      </c>
-      <c r="B230" s="7">
-        <v>4.4321248000000004</v>
-      </c>
-      <c r="C230" s="7">
         <v>3.4549782666666662</v>
-      </c>
-    </row>
-    <row r="231" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A231" t="s">
-        <v>223</v>
-      </c>
-      <c r="B231" s="7">
-        <v>-4.5080000000002896E-4</v>
-      </c>
-      <c r="C231" s="7">
-        <v>2.7959178666666671</v>
-      </c>
-    </row>
-    <row r="232" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A232" t="s">
-        <v>224</v>
-      </c>
-      <c r="B232" s="7">
-        <v>5.6353600000000059E-2</v>
-      </c>
-      <c r="C232" s="7">
-        <v>3.8036116666666677</v>
-      </c>
-    </row>
-    <row r="233" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A233" t="s">
-        <v>225</v>
-      </c>
-      <c r="B233" s="7">
-        <v>-2.9769199999999996E-2</v>
-      </c>
-      <c r="C233" s="7">
-        <v>4.4308334000000009</v>
-      </c>
-    </row>
-    <row r="234" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A234" t="s">
-        <v>226</v>
-      </c>
-      <c r="B234" s="7">
-        <v>5.0856400000000079E-2</v>
-      </c>
-      <c r="C234" s="7">
-        <v>2.7593034000000003</v>
-      </c>
-    </row>
-    <row r="235" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A235" t="s">
-        <v>227</v>
-      </c>
-      <c r="B235" s="7">
-        <v>-2.6104400000000028E-2</v>
-      </c>
-      <c r="C235" s="7">
-        <v>1.956969</v>
-      </c>
-    </row>
-    <row r="236" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A236" t="s">
-        <v>228</v>
-      </c>
-      <c r="B236" s="7">
-        <v>-4.115599999999997E-3</v>
-      </c>
-      <c r="C236" s="7">
-        <v>0.2973785000000001</v>
-      </c>
-    </row>
-    <row r="237" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A237" t="s">
-        <v>229</v>
-      </c>
-      <c r="B237" s="7">
-        <v>-1.3277600000000056E-2</v>
-      </c>
-      <c r="C237" s="7">
-        <v>9.9182800000000126E-2</v>
-      </c>
-    </row>
-    <row r="238" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A238" t="s">
-        <v>230</v>
-      </c>
-      <c r="B238" s="7">
-        <v>-4.5080000000002896E-4</v>
-      </c>
-      <c r="C238" s="7">
-        <v>3.9485300000000056E-2</v>
-      </c>
-    </row>
-    <row r="239" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A239" t="s">
-        <v>231</v>
-      </c>
-      <c r="B239" s="7">
-        <v>-2.6104399999999917E-2</v>
-      </c>
-      <c r="C239" s="7">
-        <v>9.9182799999999904E-2</v>
-      </c>
-    </row>
-    <row r="240" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A240" t="s">
-        <v>232</v>
-      </c>
-      <c r="B240" s="7">
-        <v>-1.5110000000000012E-2</v>
-      </c>
-      <c r="C240" s="7">
-        <v>0.37617920000000016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>